<commit_message>
Changed the "use_dam_level_df" to "Yes", and received the following error message when running the code: """ Field DFU does not exist Field DFD does not exist There were 2 fields missing from the table. Please fix add the fields to the table before proceeding """
Checked the documentation of GDW dataset, and other things, but could not
find any info about the "DFU" and "DFD" fields.

What about the "drf" and "dfd" fields? Are they the same as "DFU" and "DFD"?
If so, then I can change the code to use "drf" and "dfd" instead of "DFU" and "DFD".
</commit_message>
<xml_diff>
--- a/config/config.xlsx
+++ b/config/config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\GitHub\Free-Flowing-Rivers\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9EC3CF-3218-4425-B819-5105627418D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48168F3-1FA2-4AD4-8B89-B8BD35E88AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="716" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="716" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="START" sheetId="33" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="212">
   <si>
     <t>URB</t>
   </si>
@@ -548,9 +548,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>min_length</t>
   </si>
   <si>
@@ -659,9 +656,6 @@
     <t>D:\Peninsular India\Output</t>
   </si>
   <si>
-    <t>DOF_try1</t>
-  </si>
-  <si>
     <t>DOR_try1</t>
   </si>
   <si>
@@ -678,6 +672,9 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>DOF_try2</t>
   </si>
 </sst>
 </file>
@@ -1748,18 +1745,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1767,7 +1764,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>30</v>
@@ -1775,26 +1772,26 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>30</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -1826,7 +1823,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>8</v>
@@ -1835,7 +1832,7 @@
         <v>7</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -1847,7 +1844,7 @@
         <v>dams_fc</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D2" s="23" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -1863,7 +1860,7 @@
         <v>bench_fc</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D3" s="23" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -1879,7 +1876,7 @@
         <v>streams_fc</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D4" s="23" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -1895,7 +1892,7 @@
         <v>lakes_fc</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D5" s="23" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -1917,7 +1914,7 @@
         <v>output_folder</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D6" s="23" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -1933,7 +1930,7 @@
         <v>barrier_inc_field</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D7" s="27" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -1981,7 +1978,7 @@
         <v>dof_field</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="D10" s="30" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -2029,7 +2026,7 @@
         <v>use_dam_level_df</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D13" s="30" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -2061,7 +2058,7 @@
         <v>dor_field</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D15" s="33" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -2077,7 +2074,7 @@
         <v>svol_field</v>
       </c>
       <c r="C16" s="32" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D16" s="33" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -2099,7 +2096,7 @@
         <v>sed_field</v>
       </c>
       <c r="C17" s="35" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D17" s="36" t="str">
         <f>Table8[[#This Row],[Short description]]</f>
@@ -2309,7 +2306,7 @@
         <v>0</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
@@ -9454,13 +9451,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B1" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>182</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -9468,10 +9465,10 @@
         <v>163</v>
       </c>
       <c r="B2" s="43" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -9482,7 +9479,7 @@
         <v>26</v>
       </c>
       <c r="C3" s="44" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -9490,10 +9487,10 @@
         <v>163</v>
       </c>
       <c r="B4" s="43" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -9504,7 +9501,7 @@
         <v>157</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
@@ -9515,7 +9512,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="75" x14ac:dyDescent="0.25">
@@ -9526,7 +9523,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
@@ -9534,10 +9531,10 @@
         <v>165</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
@@ -9545,10 +9542,10 @@
         <v>165</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -9559,7 +9556,7 @@
         <v>6</v>
       </c>
       <c r="C10" s="47" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
@@ -9570,7 +9567,7 @@
         <v>166</v>
       </c>
       <c r="C11" s="47" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
@@ -9581,7 +9578,7 @@
         <v>167</v>
       </c>
       <c r="C12" s="47" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
@@ -9592,7 +9589,7 @@
         <v>27</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -9614,7 +9611,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -9636,7 +9633,7 @@
         <v>158</v>
       </c>
       <c r="C17" s="53" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>